<commit_message>
feat: update final execution results
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\xivqn\GitHub\TMB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABC09C0F-43DA-4702-8B50-166BE5F23984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{90790DB4-5E64-47E7-8226-2A307EA2132A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14550" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,6 +41,9 @@
     <t>IC</t>
   </si>
   <si>
+    <t>LT</t>
+  </si>
+  <si>
     <t>γ</t>
   </si>
   <si>
@@ -53,10 +56,13 @@
     <t>STMB</t>
   </si>
   <si>
+    <t>GRASP</t>
+  </si>
+  <si>
     <t>|A|</t>
   </si>
   <si>
-    <t>Dev. (%)</t>
+    <t>Dev.</t>
   </si>
   <si>
     <t>Time (s)</t>
@@ -65,15 +71,18 @@
     <t>0.02</t>
   </si>
   <si>
+    <t>as20000102</t>
+  </si>
+  <si>
     <t>Brightkite_edges</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>CA-HepTh</t>
   </si>
   <si>
-    <t>as20000102</t>
-  </si>
-  <si>
     <t>p2p-Gnutella04</t>
   </si>
   <si>
@@ -84,22 +93,13 @@
   </si>
   <si>
     <t>0.10</t>
-  </si>
-  <si>
-    <t>LT</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>GRASP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,6 +126,14 @@
       <b/>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -389,7 +397,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -436,6 +444,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -454,20 +477,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="2" fontId="4" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -751,384 +786,386 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:X16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="3" max="3" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7265625" customWidth="1"/>
-    <col min="11" max="11" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:24" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="26"/>
-      <c r="N2" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="O2" s="25"/>
-      <c r="P2" s="25"/>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-      <c r="S2" s="25"/>
-      <c r="T2" s="25"/>
-      <c r="U2" s="25"/>
-      <c r="V2" s="25"/>
-      <c r="W2" s="25"/>
-      <c r="X2" s="26"/>
+    <row r="1" spans="2:24" ht="15" thickBot="1"/>
+    <row r="2" spans="2:24" ht="15.95" thickBot="1">
+      <c r="B2" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="18"/>
+      <c r="N2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="17"/>
+      <c r="V2" s="17"/>
+      <c r="W2" s="17"/>
+      <c r="X2" s="18"/>
     </row>
-    <row r="3" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B3" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="22" t="s">
+    <row r="3" spans="2:24">
+      <c r="B3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="C3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="17"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="16" t="s">
+      <c r="D3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="17"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="17"/>
-      <c r="L3" s="18"/>
-      <c r="N3" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="O3" s="22" t="s">
+      <c r="E3" s="22"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="22"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" s="22"/>
+      <c r="L3" s="23"/>
+      <c r="N3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="P3" s="16" t="s">
+      <c r="O3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="18"/>
-      <c r="S3" s="16" t="s">
+      <c r="P3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="T3" s="17"/>
-      <c r="U3" s="18"/>
-      <c r="V3" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="W3" s="17"/>
-      <c r="X3" s="18"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="T3" s="22"/>
+      <c r="U3" s="23"/>
+      <c r="V3" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="W3" s="22"/>
+      <c r="X3" s="23"/>
     </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
+    <row r="4" spans="2:24">
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
       <c r="D4" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="R4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="S4" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="U4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="V4" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="X4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:24" ht="15">
+      <c r="B5" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="13">
+        <v>7</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="F5" s="27">
+        <v>1.97</v>
+      </c>
+      <c r="G5" s="33">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="H5" s="30">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5">
+        <v>406.44</v>
+      </c>
+      <c r="J5" s="13">
         <v>6</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="J4" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="R4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="S4" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="U4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="W4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="X4" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B5" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="13">
-        <v>136</v>
-      </c>
-      <c r="E5" s="2">
-        <v>4.9130434782608692</v>
-      </c>
-      <c r="F5" s="5">
-        <v>43.881999999999998</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" s="13">
-        <v>23</v>
-      </c>
       <c r="K5" s="2">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="L5" s="5">
-        <v>18009.624</v>
-      </c>
-      <c r="N5" s="19" t="s">
-        <v>8</v>
+        <v>1027.9000000000001</v>
+      </c>
+      <c r="N5" s="24" t="s">
+        <v>10</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P5" s="13">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="2">
-        <v>16</v>
+        <v>5.5</v>
       </c>
       <c r="R5" s="5">
-        <v>8.91</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="S5" s="13">
         <v>12</v>
       </c>
       <c r="T5" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U5" s="5">
-        <v>10519.547</v>
+        <v>766.1</v>
       </c>
       <c r="V5" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W5" s="2">
         <v>0</v>
       </c>
       <c r="X5" s="5">
-        <v>20981.360000000001</v>
+        <v>90.11</v>
       </c>
     </row>
-    <row r="6" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B6" s="19"/>
+    <row r="6" spans="2:24" ht="15">
+      <c r="B6" s="24"/>
       <c r="C6" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D6" s="14">
-        <v>87</v>
+        <v>32</v>
       </c>
       <c r="E6" s="3">
-        <v>86</v>
-      </c>
-      <c r="F6" s="6">
-        <v>2.1110000000000002</v>
-      </c>
-      <c r="G6" s="14">
-        <v>6</v>
-      </c>
-      <c r="H6" s="3">
-        <v>5</v>
-      </c>
-      <c r="I6" s="6">
-        <v>60.036000000000001</v>
-      </c>
-      <c r="J6" s="14">
-        <v>1</v>
-      </c>
-      <c r="K6" s="3">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="F6" s="28">
+        <v>245.77</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="32">
+        <v>30</v>
+      </c>
+      <c r="K6" s="31">
         <v>0</v>
       </c>
       <c r="L6" s="6">
-        <v>5.3540000000000001</v>
-      </c>
-      <c r="N6" s="19"/>
+        <v>19026.95</v>
+      </c>
+      <c r="N6" s="24"/>
       <c r="O6" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="P6" s="14">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="Q6" s="3">
         <v>16</v>
       </c>
       <c r="R6" s="6">
-        <v>0.31</v>
+        <v>8.91</v>
       </c>
       <c r="S6" s="14">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="T6" s="3">
-        <v>0</v>
+        <v>1.6666666666666667</v>
       </c>
       <c r="U6" s="6">
-        <v>71.927000000000007</v>
+        <v>3755.62</v>
       </c>
       <c r="V6" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W6" s="3">
         <v>0</v>
       </c>
       <c r="X6" s="6">
-        <v>0.05</v>
+        <v>8307.84</v>
       </c>
     </row>
-    <row r="7" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B7" s="19"/>
+    <row r="7" spans="2:24" ht="15">
+      <c r="B7" s="24"/>
       <c r="C7" s="9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D7" s="13">
-        <v>10</v>
-      </c>
-      <c r="E7" s="2">
-        <v>9</v>
-      </c>
-      <c r="F7" s="5">
-        <v>0.1</v>
+        <v>5</v>
+      </c>
+      <c r="E7" s="30">
+        <v>0</v>
+      </c>
+      <c r="F7" s="27">
+        <v>2.5499999999999998</v>
       </c>
       <c r="G7" s="13">
         <v>6</v>
       </c>
       <c r="H7" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I7" s="5">
+        <v>901.11</v>
+      </c>
+      <c r="J7" s="33">
         <v>5</v>
       </c>
-      <c r="I7" s="5">
-        <v>3.46</v>
-      </c>
-      <c r="J7" s="13">
+      <c r="K7" s="30">
+        <v>0</v>
+      </c>
+      <c r="L7" s="5">
+        <v>7447.52</v>
+      </c>
+      <c r="N7" s="24"/>
+      <c r="O7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="P7" s="13">
+        <v>17</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>16</v>
+      </c>
+      <c r="R7" s="5">
+        <v>0.31</v>
+      </c>
+      <c r="S7" s="13">
         <v>1</v>
       </c>
-      <c r="K7" s="2">
-        <v>0</v>
-      </c>
-      <c r="L7" s="5">
-        <v>126.43899999999999</v>
-      </c>
-      <c r="N7" s="19"/>
-      <c r="O7" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="P7" s="13">
-        <v>13</v>
-      </c>
-      <c r="Q7" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="R7" s="5">
-        <v>0.14899999999999999</v>
-      </c>
-      <c r="S7" s="13">
-        <v>14</v>
-      </c>
       <c r="T7" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U7" s="5">
-        <v>3.3290000000000002</v>
+        <v>317.89</v>
       </c>
       <c r="V7" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W7" s="2">
         <v>0</v>
       </c>
       <c r="X7" s="5">
-        <v>163.17699999999999</v>
+        <v>0.94</v>
       </c>
     </row>
-    <row r="8" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B8" s="19"/>
+    <row r="8" spans="2:24" ht="15">
+      <c r="B8" s="24"/>
       <c r="C8" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D8" s="14">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="E8" s="3">
-        <v>0</v>
-      </c>
-      <c r="F8" s="6">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="G8" s="14">
+        <v>13.333333333333334</v>
+      </c>
+      <c r="F8" s="28">
+        <v>4.47</v>
+      </c>
+      <c r="G8" s="32">
         <v>3</v>
       </c>
-      <c r="H8" s="3">
-        <v>2</v>
+      <c r="H8" s="31">
+        <v>0</v>
       </c>
       <c r="I8" s="6">
-        <v>6.3170000000000002</v>
+        <v>505.81</v>
       </c>
       <c r="J8" s="14">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K8" s="3">
-        <v>0</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="L8" s="6">
-        <v>45.145000000000003</v>
-      </c>
-      <c r="N8" s="19"/>
+        <v>18021.080000000002</v>
+      </c>
+      <c r="N8" s="24"/>
       <c r="O8" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="P8" s="14">
         <v>24</v>
@@ -1140,13 +1177,13 @@
         <v>0.88800000000000001</v>
       </c>
       <c r="S8" s="14">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="T8" s="3">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="U8" s="6">
-        <v>6.64</v>
+        <v>962.38</v>
       </c>
       <c r="V8" s="14">
         <v>1</v>
@@ -1155,44 +1192,44 @@
         <v>0</v>
       </c>
       <c r="X8" s="6">
-        <v>5.0000000000000001E-3</v>
+        <v>0.77</v>
       </c>
     </row>
-    <row r="9" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B9" s="19"/>
+    <row r="9" spans="2:24" ht="15">
+      <c r="B9" s="24"/>
       <c r="C9" s="9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D9" s="13">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="E9" s="2">
-        <v>18</v>
-      </c>
-      <c r="F9" s="5">
-        <v>1.35</v>
+        <v>0.5</v>
+      </c>
+      <c r="F9" s="27">
+        <v>4.67</v>
       </c>
       <c r="G9" s="13">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H9" s="2">
-        <v>2.3333333333333335</v>
+        <v>0.25</v>
       </c>
       <c r="I9" s="5">
-        <v>4.8159999999999998</v>
-      </c>
-      <c r="J9" s="13">
-        <v>3</v>
-      </c>
-      <c r="K9" s="2">
+        <v>397.08</v>
+      </c>
+      <c r="J9" s="33">
+        <v>4</v>
+      </c>
+      <c r="K9" s="30">
         <v>0</v>
       </c>
       <c r="L9" s="5">
-        <v>687.45899999999995</v>
-      </c>
-      <c r="N9" s="19"/>
+        <v>3922.34</v>
+      </c>
+      <c r="N9" s="24"/>
       <c r="O9" s="9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="P9" s="13">
         <v>51</v>
@@ -1210,7 +1247,7 @@
         <v>2.5</v>
       </c>
       <c r="U9" s="5">
-        <v>4.117</v>
+        <v>360.07</v>
       </c>
       <c r="V9" s="13">
         <v>2</v>
@@ -1219,44 +1256,44 @@
         <v>0</v>
       </c>
       <c r="X9" s="5">
-        <v>474.47199999999998</v>
+        <v>216.12</v>
       </c>
     </row>
-    <row r="10" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B10" s="19"/>
+    <row r="10" spans="2:24" ht="15">
+      <c r="B10" s="24"/>
       <c r="C10" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="14">
+        <v>50</v>
+      </c>
+      <c r="E10" s="3">
+        <v>2.5714285714285716</v>
+      </c>
+      <c r="F10" s="28">
+        <v>133.61000000000001</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="32">
         <v>14</v>
       </c>
-      <c r="D10" s="14">
-        <v>1</v>
-      </c>
-      <c r="E10" s="3">
-        <v>0</v>
-      </c>
-      <c r="F10" s="6">
-        <v>0.60699999999999998</v>
-      </c>
-      <c r="G10" s="14" t="s">
+      <c r="K10" s="31">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6">
+        <v>18653.48</v>
+      </c>
+      <c r="N10" s="24"/>
+      <c r="O10" s="10" t="s">
         <v>17</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="14">
-        <v>1</v>
-      </c>
-      <c r="K10" s="3">
-        <v>0</v>
-      </c>
-      <c r="L10" s="6">
-        <v>0.48799999999999999</v>
-      </c>
-      <c r="N10" s="19"/>
-      <c r="O10" s="10" t="s">
-        <v>14</v>
       </c>
       <c r="P10" s="14">
         <v>44</v>
@@ -1268,13 +1305,13 @@
         <v>5.6219999999999999</v>
       </c>
       <c r="S10" s="14" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="U10" s="6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="V10" s="14">
         <v>1</v>
@@ -1283,240 +1320,240 @@
         <v>0</v>
       </c>
       <c r="X10" s="6">
-        <v>741.07399999999996</v>
+        <v>525.71</v>
       </c>
     </row>
-    <row r="11" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B11" s="20" t="s">
+    <row r="11" spans="2:24" ht="15">
+      <c r="B11" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="13">
+        <v>40</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.21212121212121213</v>
+      </c>
+      <c r="F11" s="27">
+        <v>2.89</v>
+      </c>
+      <c r="G11" s="33">
+        <v>33</v>
+      </c>
+      <c r="H11" s="30">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5">
+        <v>1660.41</v>
+      </c>
+      <c r="J11" s="13">
+        <v>35</v>
+      </c>
+      <c r="K11" s="2">
+        <v>6.0606060606060608E-2</v>
+      </c>
+      <c r="L11" s="5">
+        <v>18014.54</v>
+      </c>
+      <c r="N11" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="O11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="P11" s="13">
+        <v>31</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>1.3846153846153846</v>
+      </c>
+      <c r="R11" s="5">
+        <v>0.30399999999999999</v>
+      </c>
+      <c r="S11" s="13">
+        <v>44</v>
+      </c>
+      <c r="T11" s="2">
+        <v>2.3846153846153846</v>
+      </c>
+      <c r="U11" s="5">
+        <v>1199.1500000000001</v>
+      </c>
+      <c r="V11" s="13">
+        <v>13</v>
+      </c>
+      <c r="W11" s="2">
+        <v>0</v>
+      </c>
+      <c r="X11" s="5">
+        <v>15664.68</v>
+      </c>
+    </row>
+    <row r="12" spans="2:24" ht="15">
+      <c r="B12" s="25"/>
+      <c r="C12" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="14">
+        <v>194</v>
+      </c>
+      <c r="E12" s="3">
+        <v>5.1813471502590676E-3</v>
+      </c>
+      <c r="F12" s="28">
+        <v>448.46</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J12" s="32">
+        <v>193</v>
+      </c>
+      <c r="K12" s="31">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6">
+        <v>20336.14</v>
+      </c>
+      <c r="N12" s="25"/>
+      <c r="O12" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="P12" s="14">
+        <v>157</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>6.85</v>
+      </c>
+      <c r="R12" s="6">
+        <v>30.369</v>
+      </c>
+      <c r="S12" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="T12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="U12" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="V12" s="14">
+        <v>20</v>
+      </c>
+      <c r="W12" s="3">
+        <v>0</v>
+      </c>
+      <c r="X12" s="6">
+        <v>18735.04</v>
+      </c>
+    </row>
+    <row r="13" spans="2:24" ht="15">
+      <c r="B13" s="25"/>
+      <c r="C13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="13">
+        <v>43</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0.59259259259259256</v>
+      </c>
+      <c r="F13" s="27">
+        <v>5.19</v>
+      </c>
+      <c r="G13" s="13">
+        <v>30</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="I13" s="5">
+        <v>2770.29</v>
+      </c>
+      <c r="J13" s="33">
+        <v>27</v>
+      </c>
+      <c r="K13" s="30">
+        <v>0</v>
+      </c>
+      <c r="L13" s="5">
+        <v>18021.73</v>
+      </c>
+      <c r="N13" s="25"/>
+      <c r="O13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="P13" s="13">
+        <v>125</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>40.666666666666664</v>
+      </c>
+      <c r="R13" s="5">
+        <v>1.357</v>
+      </c>
+      <c r="S13" s="13">
+        <v>13</v>
+      </c>
+      <c r="T13" s="2">
+        <v>3.3333333333333335</v>
+      </c>
+      <c r="U13" s="5">
+        <v>822.8</v>
+      </c>
+      <c r="V13" s="13">
+        <v>3</v>
+      </c>
+      <c r="W13" s="2">
+        <v>0</v>
+      </c>
+      <c r="X13" s="5">
+        <v>641.89</v>
+      </c>
+    </row>
+    <row r="14" spans="2:24" ht="15">
+      <c r="B14" s="25"/>
+      <c r="C14" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="13">
-        <v>472</v>
-      </c>
-      <c r="E11" s="2">
-        <v>1.5792349726775956</v>
-      </c>
-      <c r="F11" s="5">
-        <v>148.988</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" s="13">
-        <v>183</v>
-      </c>
-      <c r="K11" s="2">
-        <v>0</v>
-      </c>
-      <c r="L11" s="5">
-        <v>18037.620999999999</v>
-      </c>
-      <c r="N11" s="20" t="s">
+      <c r="D14" s="14">
+        <v>131</v>
+      </c>
+      <c r="E14" s="3">
+        <v>5.55</v>
+      </c>
+      <c r="F14" s="28">
+        <v>5.2</v>
+      </c>
+      <c r="G14" s="32">
+        <v>20</v>
+      </c>
+      <c r="H14" s="31">
+        <v>0</v>
+      </c>
+      <c r="I14" s="6">
+        <v>1717.32</v>
+      </c>
+      <c r="J14" s="14">
+        <v>76</v>
+      </c>
+      <c r="K14" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="L14" s="6">
+        <v>18057.36</v>
+      </c>
+      <c r="N14" s="25"/>
+      <c r="O14" s="10" t="s">
         <v>15</v>
-      </c>
-      <c r="O11" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="P11" s="13">
-        <v>157</v>
-      </c>
-      <c r="Q11" s="2">
-        <v>9.4666666666666668</v>
-      </c>
-      <c r="R11" s="5">
-        <v>30.369</v>
-      </c>
-      <c r="S11" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="T11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="V11" s="13">
-        <v>15</v>
-      </c>
-      <c r="W11" s="2">
-        <v>0</v>
-      </c>
-      <c r="X11" s="5">
-        <v>18001.968000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B12" s="20"/>
-      <c r="C12" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="14">
-        <v>169</v>
-      </c>
-      <c r="E12" s="3">
-        <v>6.041666666666667</v>
-      </c>
-      <c r="F12" s="6">
-        <v>4.5359999999999996</v>
-      </c>
-      <c r="G12" s="14">
-        <v>46</v>
-      </c>
-      <c r="H12" s="3">
-        <v>0.91666666666666663</v>
-      </c>
-      <c r="I12" s="6">
-        <v>58.682000000000002</v>
-      </c>
-      <c r="J12" s="14">
-        <v>24</v>
-      </c>
-      <c r="K12" s="3">
-        <v>0</v>
-      </c>
-      <c r="L12" s="6">
-        <v>18860.879000000001</v>
-      </c>
-      <c r="N12" s="20"/>
-      <c r="O12" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="P12" s="14">
-        <v>125</v>
-      </c>
-      <c r="Q12" s="3">
-        <v>40.666666666666664</v>
-      </c>
-      <c r="R12" s="6">
-        <v>1.357</v>
-      </c>
-      <c r="S12" s="14">
-        <v>18</v>
-      </c>
-      <c r="T12" s="3">
-        <v>5</v>
-      </c>
-      <c r="U12" s="6">
-        <v>69.486999999999995</v>
-      </c>
-      <c r="V12" s="14">
-        <v>3</v>
-      </c>
-      <c r="W12" s="3">
-        <v>0</v>
-      </c>
-      <c r="X12" s="6">
-        <v>231.63900000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B13" s="20"/>
-      <c r="C13" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="13">
-        <v>37</v>
-      </c>
-      <c r="E13" s="2">
-        <v>0.27586206896551724</v>
-      </c>
-      <c r="F13" s="5">
-        <v>0.36399999999999999</v>
-      </c>
-      <c r="G13" s="13">
-        <v>33</v>
-      </c>
-      <c r="H13" s="2">
-        <v>0.13793103448275862</v>
-      </c>
-      <c r="I13" s="5">
-        <v>3.532</v>
-      </c>
-      <c r="J13" s="13">
-        <v>29</v>
-      </c>
-      <c r="K13" s="2">
-        <v>0</v>
-      </c>
-      <c r="L13" s="5">
-        <v>18362.595000000001</v>
-      </c>
-      <c r="N13" s="20"/>
-      <c r="O13" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="P13" s="13">
-        <v>31</v>
-      </c>
-      <c r="Q13" s="2">
-        <v>1.3846153846153846</v>
-      </c>
-      <c r="R13" s="5">
-        <v>0.30399999999999999</v>
-      </c>
-      <c r="S13" s="13">
-        <v>61</v>
-      </c>
-      <c r="T13" s="2">
-        <v>3.6923076923076925</v>
-      </c>
-      <c r="U13" s="5">
-        <v>3.4550000000000001</v>
-      </c>
-      <c r="V13" s="13">
-        <v>13</v>
-      </c>
-      <c r="W13" s="2">
-        <v>0</v>
-      </c>
-      <c r="X13" s="5">
-        <v>6391.6750000000002</v>
-      </c>
-    </row>
-    <row r="14" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B14" s="20"/>
-      <c r="C14" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="14">
-        <v>130</v>
-      </c>
-      <c r="E14" s="3">
-        <v>5.1904761904761907</v>
-      </c>
-      <c r="F14" s="6">
-        <v>0.64700000000000002</v>
-      </c>
-      <c r="G14" s="14">
-        <v>21</v>
-      </c>
-      <c r="H14" s="3">
-        <v>0</v>
-      </c>
-      <c r="I14" s="6">
-        <v>6.58</v>
-      </c>
-      <c r="J14" s="14">
-        <v>98</v>
-      </c>
-      <c r="K14" s="3">
-        <v>3.6665999999999999</v>
-      </c>
-      <c r="L14" s="6">
-        <v>18013.240000000002</v>
-      </c>
-      <c r="N14" s="20"/>
-      <c r="O14" s="10" t="s">
-        <v>12</v>
       </c>
       <c r="P14" s="14">
         <v>74</v>
@@ -1528,13 +1565,13 @@
         <v>2.0870000000000002</v>
       </c>
       <c r="S14" s="14">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="T14" s="3">
-        <v>32.5</v>
+        <v>36.5</v>
       </c>
       <c r="U14" s="6">
-        <v>6.9089999999999998</v>
+        <v>3710.71</v>
       </c>
       <c r="V14" s="14">
         <v>2</v>
@@ -1543,44 +1580,44 @@
         <v>0</v>
       </c>
       <c r="X14" s="6">
-        <v>572.87</v>
+        <v>2384.7800000000002</v>
       </c>
     </row>
-    <row r="15" spans="2:24" x14ac:dyDescent="0.35">
-      <c r="B15" s="20"/>
+    <row r="15" spans="2:24" ht="15">
+      <c r="B15" s="25"/>
       <c r="C15" s="9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D15" s="13">
-        <v>113</v>
+        <v>29</v>
       </c>
       <c r="E15" s="2">
-        <v>3.3461538461538463</v>
-      </c>
-      <c r="F15" s="5">
-        <v>3.278</v>
+        <v>3.5714285714285712E-2</v>
+      </c>
+      <c r="F15" s="27">
+        <v>5.58</v>
       </c>
       <c r="G15" s="13">
-        <v>291</v>
+        <v>29</v>
       </c>
       <c r="H15" s="2">
-        <v>10.192307692307692</v>
+        <v>3.5714285714285712E-2</v>
       </c>
       <c r="I15" s="5">
-        <v>8.1630000000000003</v>
-      </c>
-      <c r="J15" s="13">
-        <v>26</v>
-      </c>
-      <c r="K15" s="2">
+        <v>1233.1400000000001</v>
+      </c>
+      <c r="J15" s="33">
+        <v>28</v>
+      </c>
+      <c r="K15" s="30">
         <v>0</v>
       </c>
       <c r="L15" s="5">
-        <v>18726.879000000001</v>
-      </c>
-      <c r="N15" s="20"/>
+        <v>18026.2</v>
+      </c>
+      <c r="N15" s="25"/>
       <c r="O15" s="9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="P15" s="13">
         <v>97</v>
@@ -1592,13 +1629,13 @@
         <v>2.173</v>
       </c>
       <c r="S15" s="13">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="T15" s="2">
-        <v>2</v>
+        <v>2.1818181818181817</v>
       </c>
       <c r="U15" s="5">
-        <v>4.0999999999999996</v>
+        <v>1005.73</v>
       </c>
       <c r="V15" s="13">
         <v>11</v>
@@ -1607,71 +1644,71 @@
         <v>0</v>
       </c>
       <c r="X15" s="5">
-        <v>5338.4790000000003</v>
+        <v>15951.33</v>
       </c>
     </row>
-    <row r="16" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="21"/>
+    <row r="16" spans="2:24" ht="15">
+      <c r="B16" s="26"/>
       <c r="C16" s="11" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D16" s="15">
-        <v>218</v>
+        <v>408</v>
       </c>
       <c r="E16" s="7">
-        <v>1.2244897959183674</v>
-      </c>
-      <c r="F16" s="8">
-        <v>79.912999999999997</v>
+        <v>0.7361702127659574</v>
+      </c>
+      <c r="F16" s="29">
+        <v>386.46</v>
       </c>
       <c r="G16" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="J16" s="34">
+        <v>235</v>
+      </c>
+      <c r="K16" s="35">
+        <v>0</v>
+      </c>
+      <c r="L16" s="8">
+        <v>19794.05</v>
+      </c>
+      <c r="N16" s="26"/>
+      <c r="O16" s="11" t="s">
         <v>17</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" s="15">
-        <v>98</v>
-      </c>
-      <c r="K16" s="7">
-        <v>0</v>
-      </c>
-      <c r="L16" s="8">
-        <v>18024.126</v>
-      </c>
-      <c r="N16" s="21"/>
-      <c r="O16" s="11" t="s">
-        <v>14</v>
       </c>
       <c r="P16" s="15">
         <v>123</v>
       </c>
       <c r="Q16" s="7">
-        <v>4.125</v>
+        <v>4.3478260869565215</v>
       </c>
       <c r="R16" s="8">
         <v>17.384</v>
       </c>
       <c r="S16" s="15" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="T16" s="7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="U16" s="8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="V16" s="15">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="W16" s="7">
         <v>0</v>
       </c>
       <c r="X16" s="8">
-        <v>18002.037</v>
+        <v>18611.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>